<commit_message>
feat: atualizacao completa do app.py com todas as 7 abas, kanban estruturado e persistencia de usuarios
</commit_message>
<xml_diff>
--- a/logs_auditoria_sistema.xlsx
+++ b/logs_auditoria_sistema.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mribeiro1\MARINGA TURISMO\Maringá Turismo - PLANEJAMENTO ESTRATEGICO (1)\01-Planejamento Estratégico\Ferramenta de Controle - Compliance\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE93B98-1E6F-4AB5-9639-2F9E09B6388E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Data_Hora</t>
   </si>
@@ -27,135 +33,12 @@
   <si>
     <t>Detalhe</t>
   </si>
-  <si>
-    <t>2026-09-04 16:01:02</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:01:24</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:01:51</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:03:01</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:32:14</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:32:22</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:32:24</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:33:27</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:57:53</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:58:17</t>
-  </si>
-  <si>
-    <t>2026-09-04 16:58:22</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:04:23</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:07:05</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:09:28</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:13:14</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:14:23</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:14:33</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:14:51</t>
-  </si>
-  <si>
-    <t>2026-09-04 17:14:59</t>
-  </si>
-  <si>
-    <t>2026-09-11 12:02:27</t>
-  </si>
-  <si>
-    <t>mribeiro1</t>
-  </si>
-  <si>
-    <t>Login</t>
-  </si>
-  <si>
-    <t>Mover Status</t>
-  </si>
-  <si>
-    <t>Inclusão</t>
-  </si>
-  <si>
-    <t>Upload Evidência</t>
-  </si>
-  <si>
-    <t>Mover Card</t>
-  </si>
-  <si>
-    <t>Evidência</t>
-  </si>
-  <si>
-    <t>Comentário</t>
-  </si>
-  <si>
-    <t>Autenticação realizada com sucesso</t>
-  </si>
-  <si>
-    <t>Alterou AUD-01 para Em Validação</t>
-  </si>
-  <si>
-    <t>Criou o apontamento AUD-05</t>
-  </si>
-  <si>
-    <t>Anexou AUD-01_Captura de tela 2026-09-03 170329.png ao ID AUD-01</t>
-  </si>
-  <si>
-    <t>Autenticação bem-sucedida</t>
-  </si>
-  <si>
-    <t>Moveu AUD-02 para A Fazer</t>
-  </si>
-  <si>
-    <t>Moveu AUD-04 para A Fazer</t>
-  </si>
-  <si>
-    <t>Atualizou evidência do AUD-01</t>
-  </si>
-  <si>
-    <t>Autenticação realizada</t>
-  </si>
-  <si>
-    <t>Comentou no card AUD-02</t>
-  </si>
-  <si>
-    <t>Acesso realizado</t>
-  </si>
-  <si>
-    <t>Acesso efetuado</t>
-  </si>
-  <si>
-    <t>Criou AUD-05</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,13 +75,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -236,7 +127,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -270,6 +161,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -304,9 +196,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -479,11 +372,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -497,292 +396,21 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" t="s">
-        <v>25</v>
-      </c>
-      <c r="D21" t="s">
-        <v>43</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100679A9D6214E23F41806BF79AA97D961D" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="615285cd3b9bba93d383710380480058">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c6f2750a-443f-47f1-aeea-95bbc8068025" xmlns:ns3="06f4cf46-f048-460d-8a19-e2350c45d0c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="450288bfee094da864ded7851c9db2e7" ns2:_="" ns3:_="">
     <xsd:import namespace="c6f2750a-443f-47f1-aeea-95bbc8068025"/>
@@ -995,15 +623,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1016,13 +635,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F06395F-31CD-48F8-AC88-9DBB5FF9FF3F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{551C3AEC-CC0E-46EB-B1DE-03C3CA564288}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{551C3AEC-CC0E-46EB-B1DE-03C3CA564288}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F06395F-31CD-48F8-AC88-9DBB5FF9FF3F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c6f2750a-443f-47f1-aeea-95bbc8068025"/>
+    <ds:schemaRef ds:uri="06f4cf46-f048-460d-8a19-e2350c45d0c5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95457020-2C01-4676-81D3-C07B3E27EFB5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95457020-2C01-4676-81D3-C07B3E27EFB5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="06f4cf46-f048-460d-8a19-e2350c45d0c5"/>
+    <ds:schemaRef ds:uri="c6f2750a-443f-47f1-aeea-95bbc8068025"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>